<commit_message>
Reglas base de diagnóstico basadas en literatura técnica
- 15 diagnósticos (17 filas) para gasolina en ralentí: combustión correcta,
  catalizador, mezcla rica/muy rica/ligeramente rica, pobre/ligeramente pobre,
  falla de encendido, falla por mezcla pobre, compresión/aceite, CO y O2 altos,
  muestra diluida, CO2 bajo y NOx alto
- Reemplazan las reglas de ejemplo y los códigos inventados E01/E02
- Filas con el mismo diagnóstico funcionan como alternativas (se muestra una vez)
- docs/REGLAS.md con valores de referencia, fundamento, validación y fuentes
- Pruebas con 14 casos típicos, incluido el ejemplo del Excel del cliente

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantilla/reglas_ejemplo.xlsx
+++ b/plantilla/reglas_ejemplo.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R18"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -496,7 +496,7 @@
         <v>100</v>
       </c>
       <c r="G2">
-        <v>14</v>
+        <v>12.5</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -504,8 +504,8 @@
       <c r="I2" t="str">
         <v/>
       </c>
-      <c r="J2">
-        <v>1</v>
+      <c r="J2" t="str">
+        <v/>
       </c>
       <c r="K2" t="str">
         <v/>
@@ -523,7 +523,7 @@
         <v>Combustión correcta</v>
       </c>
       <c r="P2" t="str">
-        <v>Valores dentro de los rangos normales para un motor a gasolina en buen estado.</v>
+        <v>Mezcla estequiométrica (λ ≈ 1), CO₂ alto y CO, HC y O₂ bajos: el motor quema bien y el catalizador convierte los gases.</v>
       </c>
       <c r="Q2" t="str">
         <v>No se requiere intervención. Mantener el plan de mantenimiento preventivo.</v>
@@ -540,19 +540,19 @@
         <v/>
       </c>
       <c r="C3">
-        <v>1.5</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
+        <v>0.51</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
       </c>
       <c r="E3" t="str">
         <v/>
       </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v/>
+      <c r="F3">
+        <v>400</v>
+      </c>
+      <c r="G3">
+        <v>12</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -560,8 +560,8 @@
       <c r="I3" t="str">
         <v/>
       </c>
-      <c r="J3">
-        <v>1</v>
+      <c r="J3" t="str">
+        <v/>
       </c>
       <c r="K3" t="str">
         <v/>
@@ -569,23 +569,23 @@
       <c r="L3" t="str">
         <v/>
       </c>
-      <c r="M3" t="str">
-        <v/>
+      <c r="M3">
+        <v>0.97</v>
       </c>
       <c r="N3">
-        <v>0.97</v>
+        <v>1.03</v>
       </c>
       <c r="O3" t="str">
-        <v>Mezcla rica (exceso de combustible)</v>
+        <v>Catalizador con baja eficiencia</v>
       </c>
       <c r="P3" t="str">
-        <v>Inyectores goteando; presión de combustible alta; sensor de oxígeno, MAP o temperatura defectuoso; filtro de aire obstruido.</v>
+        <v>La mezcla es correcta (λ ≈ 1) y la combustión eficiente (CO₂ normal), pero salen CO o HC por encima de lo esperado: el catalizador no está convirtiendo los gases (desgastado, contaminado por aceite o anticongelante, o no alcanza su temperatura). En vehículos sin catalizador estos valores pueden ser normales.</v>
       </c>
       <c r="Q3" t="str">
-        <v>Revisar presión de combustible y regulador, probar inyectores, verificar sensores con escáner y cambiar filtro de aire.</v>
+        <v>Verificar que el vehículo tenga catalizador y que el motor esté caliente. Medir la temperatura a la entrada y salida del catalizador (la salida debe estar más caliente). Si no convierte, reemplazarlo y corregir la causa (consumo de aceite, fallas de encendido).</v>
       </c>
       <c r="R3" t="str">
-        <v>Alta</v>
+        <v>Media</v>
       </c>
     </row>
     <row r="4">
@@ -601,20 +601,20 @@
       <c r="D4">
         <v>0.5</v>
       </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v/>
+      <c r="E4">
+        <v>101</v>
+      </c>
+      <c r="F4">
+        <v>400</v>
+      </c>
+      <c r="G4">
+        <v>12</v>
       </c>
       <c r="H4" t="str">
         <v/>
       </c>
-      <c r="I4">
-        <v>2</v>
+      <c r="I4" t="str">
+        <v/>
       </c>
       <c r="J4" t="str">
         <v/>
@@ -626,19 +626,19 @@
         <v/>
       </c>
       <c r="M4">
-        <v>1.05</v>
-      </c>
-      <c r="N4" t="str">
-        <v/>
+        <v>0.97</v>
+      </c>
+      <c r="N4">
+        <v>1.03</v>
       </c>
       <c r="O4" t="str">
-        <v>Mezcla pobre (falta de combustible o exceso de aire)</v>
+        <v>Catalizador con baja eficiencia</v>
       </c>
       <c r="P4" t="str">
-        <v>Entrada de aire falso (fuga de vacío); inyectores sucios; bomba de combustible débil; sensor MAF sucio.</v>
+        <v>La mezcla es correcta (λ ≈ 1) y la combustión eficiente (CO₂ normal), pero salen CO o HC por encima de lo esperado: el catalizador no está convirtiendo los gases (desgastado, contaminado por aceite o anticongelante, o no alcanza su temperatura). En vehículos sin catalizador estos valores pueden ser normales.</v>
       </c>
       <c r="Q4" t="str">
-        <v>Buscar fugas de vacío, limpiar inyectores y MAF, medir presión y caudal de la bomba de combustible.</v>
+        <v>Verificar que el vehículo tenga catalizador y que el motor esté caliente. Medir la temperatura a la entrada y salida del catalizador (la salida debe estar más caliente). Si no convierte, reemplazarlo y corregir la causa (consumo de aceite, fallas de encendido).</v>
       </c>
       <c r="R4" t="str">
         <v>Media</v>
@@ -651,14 +651,14 @@
       <c r="B5" t="str">
         <v/>
       </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5">
-        <v>500</v>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>2.99</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -669,8 +669,8 @@
       <c r="H5" t="str">
         <v/>
       </c>
-      <c r="I5">
-        <v>2</v>
+      <c r="I5" t="str">
+        <v/>
       </c>
       <c r="J5" t="str">
         <v/>
@@ -684,20 +684,20 @@
       <c r="M5" t="str">
         <v/>
       </c>
-      <c r="N5" t="str">
-        <v/>
+      <c r="N5">
+        <v>0.97</v>
       </c>
       <c r="O5" t="str">
-        <v>Falla de encendido (cilindro que no quema)</v>
+        <v>Mezcla rica</v>
       </c>
       <c r="P5" t="str">
-        <v>Bujías gastadas o sucias; cables de bujía o bobinas defectuosas; baja compresión en un cilindro.</v>
+        <v>Exceso de combustible: CO alto con O₂ bajo. Posibles causas: sensor de oxígeno sesgado o lento, sensor de temperatura del refrigerante indicando motor frío, presión de combustible alta (regulador), inyectores goteando, canister EVAP saturado, válvula PCV obstruida, filtro de aire sucio (motores con sensor MAP).</v>
       </c>
       <c r="Q5" t="str">
-        <v>Revisar bujías, cables y bobinas; hacer prueba de compresión si persiste.</v>
+        <v>Revisar con escáner los ajustes de combustible (fuel trims) y los sensores de O₂, ECT y MAP/MAF. Medir la presión de combustible y probar el regulador e inyectores. Revisar PCV, canister y filtro de aire.</v>
       </c>
       <c r="R5" t="str">
-        <v>Alta</v>
+        <v>Media</v>
       </c>
     </row>
     <row r="6">
@@ -707,8 +707,8 @@
       <c r="B6" t="str">
         <v/>
       </c>
-      <c r="C6" t="str">
-        <v/>
+      <c r="C6">
+        <v>3</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -722,11 +722,11 @@
       <c r="G6" t="str">
         <v/>
       </c>
-      <c r="H6">
-        <v>10</v>
-      </c>
-      <c r="I6">
-        <v>4</v>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -740,20 +740,20 @@
       <c r="M6" t="str">
         <v/>
       </c>
-      <c r="N6" t="str">
-        <v/>
+      <c r="N6">
+        <v>0.97</v>
       </c>
       <c r="O6" t="str">
-        <v>Dilución de la muestra (fuga en el escape o sonda mal colocada)</v>
+        <v>Mezcla muy rica</v>
       </c>
       <c r="P6" t="str">
-        <v>Fisura o empaque dañado en el sistema de escape; sonda del analizador insertada de forma insuficiente.</v>
+        <v>Gran exceso de combustible (CO muy alto con O₂ bajo): inyector goteando o pegado abierto, regulador de presión dañado, sensor ECT o de O₂ defectuoso, combustible en el aceite del cárter. En carburados: flotador hundido o chiclé desgastado.</v>
       </c>
       <c r="Q6" t="str">
-        <v>Verificar la inserción de la sonda (mínimo 30 cm) y revisar el escape en busca de fugas antes de repetir la prueba.</v>
+        <v>Corregir de inmediato: consume combustible en exceso y daña el catalizador. Medir presión de combustible, probar estanqueidad de inyectores, revisar sensores con escáner y oler el aceite por dilución con gasolina (cambiarlo si está contaminado).</v>
       </c>
       <c r="R6" t="str">
-        <v>Media</v>
+        <v>Alta</v>
       </c>
     </row>
     <row r="7">
@@ -763,17 +763,17 @@
       <c r="B7" t="str">
         <v/>
       </c>
-      <c r="C7">
-        <v>0.5</v>
+      <c r="C7" t="str">
+        <v/>
       </c>
       <c r="D7">
-        <v>1.5</v>
-      </c>
-      <c r="E7">
-        <v>100</v>
+        <v>0.99</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
       </c>
       <c r="F7">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G7" t="str">
         <v/>
@@ -781,8 +781,8 @@
       <c r="H7" t="str">
         <v/>
       </c>
-      <c r="I7" t="str">
-        <v/>
+      <c r="I7">
+        <v>2</v>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -793,20 +793,20 @@
       <c r="L7" t="str">
         <v/>
       </c>
-      <c r="M7">
-        <v>0.97</v>
-      </c>
-      <c r="N7">
-        <v>1.03</v>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
       </c>
       <c r="O7" t="str">
-        <v>Catalizador con baja eficiencia</v>
+        <v>Mezcla pobre</v>
       </c>
       <c r="P7" t="str">
-        <v>Mezcla correcta (lambda ≈ 1) pero CO y HC por encima de lo esperado: el catalizador no está convirtiendo los gases.</v>
+        <v>Falta de combustible o exceso de aire: O₂ alto con CO bajo. Posibles causas: entrada de aire falso (fuga de vacío, mangueras, empaque del múltiple de admisión), inyectores obstruidos, presión o caudal de combustible bajos, sensor MAF sucio.</v>
       </c>
       <c r="Q7" t="str">
-        <v>Medir temperatura de entrada y salida del catalizador; considerar su reemplazo.</v>
+        <v>Buscar fugas de vacío (prueba de humo o con limpiador de carburador y RPM), limpiar inyectores y sensor MAF, medir presión y caudal de la bomba de combustible y revisar el filtro de combustible.</v>
       </c>
       <c r="R7" t="str">
         <v>Media</v>
@@ -814,7 +814,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>R07</v>
+        <v>R06B</v>
       </c>
       <c r="B8" t="str">
         <v/>
@@ -822,14 +822,14 @@
       <c r="C8" t="str">
         <v/>
       </c>
-      <c r="D8" t="str">
-        <v/>
+      <c r="D8">
+        <v>0.99</v>
       </c>
       <c r="E8" t="str">
         <v/>
       </c>
-      <c r="F8" t="str">
-        <v/>
+      <c r="F8">
+        <v>299</v>
       </c>
       <c r="G8" t="str">
         <v/>
@@ -843,26 +843,26 @@
       <c r="J8" t="str">
         <v/>
       </c>
-      <c r="K8">
-        <v>1000</v>
+      <c r="K8" t="str">
+        <v/>
       </c>
       <c r="L8" t="str">
         <v/>
       </c>
-      <c r="M8" t="str">
-        <v/>
+      <c r="M8">
+        <v>1.05</v>
       </c>
       <c r="N8" t="str">
         <v/>
       </c>
       <c r="O8" t="str">
-        <v>NOx elevado (temperatura de combustión alta)</v>
+        <v>Mezcla pobre</v>
       </c>
       <c r="P8" t="str">
-        <v>Válvula EGR obstruida o inoperante; mezcla pobre; exceso de carbonilla; sistema de enfriamiento deficiente.</v>
+        <v>Falta de combustible o exceso de aire: O₂ alto con CO bajo. Posibles causas: entrada de aire falso (fuga de vacío, mangueras, empaque del múltiple de admisión), inyectores obstruidos, presión o caudal de combustible bajos, sensor MAF sucio.</v>
       </c>
       <c r="Q8" t="str">
-        <v>Revisar y limpiar la válvula EGR, descarbonizar el motor y verificar el sistema de enfriamiento.</v>
+        <v>Buscar fugas de vacío (prueba de humo o con limpiador de carburador y RPM), limpiar inyectores y sensor MAF, medir presión y caudal de la bomba de combustible y revisar el filtro de combustible.</v>
       </c>
       <c r="R8" t="str">
         <v>Media</v>
@@ -870,16 +870,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>R08</v>
+        <v>R07</v>
       </c>
       <c r="B9" t="str">
         <v/>
       </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9">
-        <v>1</v>
+      <c r="C9">
+        <v>0.5</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
       </c>
       <c r="E9">
         <v>300</v>
@@ -893,12 +893,12 @@
       <c r="H9" t="str">
         <v/>
       </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
-      <c r="J9">
+      <c r="I9">
         <v>2</v>
       </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
       <c r="K9" t="str">
         <v/>
       </c>
@@ -912,13 +912,13 @@
         <v/>
       </c>
       <c r="O9" t="str">
-        <v>Posible consumo de aceite</v>
+        <v>Falla de encendido (cilindro que no quema)</v>
       </c>
       <c r="P9" t="str">
-        <v>HC alto sin exceso de combustible ni de oxígeno: anillos de pistón o guías de válvula desgastados; válvula PCV defectuosa.</v>
+        <v>HC muy alto junto con O₂ y CO altos: un cilindro no quema la mezcla y sale combustible crudo; la computadora interpreta el oxígeno sobrante como mezcla pobre y enriquece. Posibles causas: bujías gastadas o sucias, cables o bobinas defectuosos, inyector de ese cilindro sin pulverizar.</v>
       </c>
       <c r="Q9" t="str">
-        <v>Revisar la válvula PCV, hacer prueba de compresión seca y húmeda, y verificar el consumo de aceite.</v>
+        <v>Revisar con escáner los contadores de fallas por cilindro (misfire). Inspeccionar bujías, cables y bobinas; intercambiar bobinas entre cilindros para ubicar la falla. Si persiste, prueba de compresión.</v>
       </c>
       <c r="R9" t="str">
         <v>Alta</v>
@@ -926,19 +926,19 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>R09</v>
+        <v>R07B</v>
       </c>
       <c r="B10" t="str">
-        <v>E01</v>
-      </c>
-      <c r="C10" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="C10">
+        <v>1.51</v>
       </c>
       <c r="D10" t="str">
         <v/>
       </c>
-      <c r="E10" t="str">
-        <v/>
+      <c r="E10">
+        <v>300</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -949,8 +949,8 @@
       <c r="H10" t="str">
         <v/>
       </c>
-      <c r="I10" t="str">
-        <v/>
+      <c r="I10">
+        <v>1</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -968,84 +968,476 @@
         <v/>
       </c>
       <c r="O10" t="str">
-        <v>Flujo de muestra bajo (código de ejemplo)</v>
+        <v>Falla de encendido (cilindro que no quema)</v>
       </c>
       <c r="P10" t="str">
-        <v>Filtro de la sonda obstruido o manguera doblada.</v>
+        <v>HC muy alto junto con O₂ y CO altos: un cilindro no quema la mezcla y sale combustible crudo; la computadora interpreta el oxígeno sobrante como mezcla pobre y enriquece. Posibles causas: bujías gastadas o sucias, cables o bobinas defectuosos, inyector de ese cilindro sin pulverizar.</v>
       </c>
       <c r="Q10" t="str">
-        <v>Limpiar o cambiar el filtro de la sonda y repetir la medición. Reemplace este código por el que imprime su equipo.</v>
+        <v>Revisar con escáner los contadores de fallas por cilindro (misfire). Inspeccionar bujías, cables y bobinas; intercambiar bobinas entre cilindros para ubicar la falla. Si persiste, prueba de compresión.</v>
       </c>
       <c r="R10" t="str">
-        <v>Media</v>
+        <v>Alta</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>R08</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11">
+        <v>0.49</v>
+      </c>
+      <c r="E11">
+        <v>300</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11">
+        <v>2</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v>Falla por mezcla muy pobre</v>
+      </c>
+      <c r="P11" t="str">
+        <v>HC alto con O₂ muy alto y CO muy bajo: la mezcla es tan pobre que la llama no la quema por completo (falla por mezcla pobre). Posibles causas: fuga de vacío grande, inyectores obstruidos, presión de combustible muy baja, sensor MAF defectuoso.</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>Buscar fugas de vacío grandes, medir presión y caudal de combustible, limpiar o probar inyectores y el sensor MAF. Verificar también que la sonda del analizador no tome aire (ver muestra diluida).</v>
+      </c>
+      <c r="R11" t="str">
+        <v>Alta</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>R09</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12">
+        <v>1.5</v>
+      </c>
+      <c r="E12">
+        <v>300</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12">
+        <v>1.99</v>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v>HC alto sin problema de mezcla: compresión, aceite o puesta a punto</v>
+      </c>
+      <c r="P12" t="str">
+        <v>Mezcla normal (ni CO ni O₂ altos) pero HC alto: el combustible no termina de quemarse por baja compresión (anillos, válvulas quemadas o mal asentadas), paso de aceite a la cámara (guías o sellos de válvula, anillos), válvula EGR abierta en ralentí o avance de encendido excesivo.</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>Hacer prueba de compresión seca y húmeda o de fugas de cilindro, revisar humo azul y consumo de aceite, verificar que la EGR cierre en ralentí y comprobar el avance de encendido.</v>
+      </c>
+      <c r="R12" t="str">
+        <v>Media</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v>R10</v>
       </c>
-      <c r="B11" t="str">
-        <v>E02</v>
-      </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11" t="str">
-        <v/>
-      </c>
-      <c r="F11" t="str">
-        <v/>
-      </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
-      <c r="H11" t="str">
-        <v/>
-      </c>
-      <c r="I11" t="str">
-        <v/>
-      </c>
-      <c r="J11" t="str">
-        <v/>
-      </c>
-      <c r="K11" t="str">
-        <v/>
-      </c>
-      <c r="L11" t="str">
-        <v/>
-      </c>
-      <c r="M11" t="str">
-        <v/>
-      </c>
-      <c r="N11" t="str">
-        <v/>
-      </c>
-      <c r="O11" t="str">
-        <v>Motor sin temperatura de operación (código de ejemplo)</v>
-      </c>
-      <c r="P11" t="str">
-        <v>La prueba se inició con el motor frío; los valores medidos no son representativos.</v>
-      </c>
-      <c r="Q11" t="str">
-        <v>Calentar el motor hasta 80 °C y repetir la prueba. Reemplace este código por el que imprime su equipo.</v>
-      </c>
-      <c r="R11" t="str">
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13">
+        <v>299</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13">
+        <v>2</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v>CO y O₂ altos a la vez</v>
+      </c>
+      <c r="P13" t="str">
+        <v>En una combustión normal no pueden estar ambos altos. Indica aire que entra al escape antes de la sonda de oxígeno (fuga en múltiple o tubo de escape), sistema de inyección de aire secundario activo, o mezcla desigual entre cilindros (un inyector goteando y otro obstruido).</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>Revisar fugas en el múltiple y el tubo de escape antes de la sonda de O₂, verificar el sistema de aire secundario si lo tiene, y hacer prueba de balance de inyectores.</v>
+      </c>
+      <c r="R13" t="str">
+        <v>Media</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>R11</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14">
+        <v>300</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14">
+        <v>10</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v>Muestra diluida: prueba no válida</v>
+      </c>
+      <c r="P14" t="str">
+        <v>CO₂ muy bajo con O₂ alto y HC normal: el analizador está midiendo aire mezclado con los gases. Sonda insertada poco profundo, fuga en el sistema de escape, o manguera o filtro del analizador con fugas.</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>Insertar la sonda al menos 30 cm dentro del tubo de escape, revisar fugas del escape y de la manguera del analizador, y repetir la medición antes de interpretar los demás resultados.</v>
+      </c>
+      <c r="R14" t="str">
+        <v>Alta</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>R12</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15">
+        <v>12.49</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15">
+        <v>0.97</v>
+      </c>
+      <c r="N15">
+        <v>1.03</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Combustión ineficiente (CO₂ bajo)</v>
+      </c>
+      <c r="P15" t="str">
+        <v>Mezcla correcta pero CO₂ bajo: la combustión no es completa. Posibles causas: puesta a punto incorrecta (avance), válvula EGR abierta en ralentí, baja compresión, o analizador descalibrado o con fugas en la sonda.</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>Verificar el avance de encendido y la EGR, hacer prueba de compresión y comprobar la calibración del analizador.</v>
+      </c>
+      <c r="R15" t="str">
+        <v>Media</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>R13</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16">
+        <v>1000</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v>NOx elevado (temperatura de combustión alta)</v>
+      </c>
+      <c r="P16" t="str">
+        <v>Temperatura o presión de combustión excesivas: válvula EGR obstruida o inoperante, mezcla pobre, avance de encendido excesivo, carbonilla en pistones o válvulas, sistema de enfriamiento deficiente, combustible de bajo octanaje o sensor de detonación inoperante.</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>Revisar y limpiar la válvula EGR y sus conductos, verificar el avance de encendido y el sensor de detonación, descarbonizar el motor y revisar el sistema de enfriamiento.</v>
+      </c>
+      <c r="R16" t="str">
+        <v>Media</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>R14</v>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17">
+        <v>300</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17">
+        <v>1.031</v>
+      </c>
+      <c r="N17">
+        <v>1.049</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Mezcla ligeramente pobre</v>
+      </c>
+      <c r="P17" t="str">
+        <v>Lambda algo por encima de 1. Puede ser la oscilación normal del control de mezcla en el momento de la medición, o una pequeña entrada de aire falso, inyectores algo sucios o un sensor de oxígeno lento.</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>Repetir la medición con el motor estabilizado. Si se mantiene, revisar con escáner los ajustes de combustible (fuel trims) y buscar pequeñas fugas de vacío.</v>
+      </c>
+      <c r="R17" t="str">
+        <v>Baja</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>R15</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18">
+        <v>0.99</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18">
+        <v>1.5</v>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18">
+        <v>0.95</v>
+      </c>
+      <c r="N18">
+        <v>0.969</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Mezcla ligeramente rica</v>
+      </c>
+      <c r="P18" t="str">
+        <v>Lambda algo por debajo de 1. Puede ser la oscilación normal del control de mezcla, o un leve exceso de combustible: sensor de oxígeno lento, filtro de aire sucio o canister EVAP purgando.</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>Repetir la medición con el motor estabilizado. Si se mantiene, revisar con escáner los ajustes de combustible, el sensor de oxígeno y el filtro de aire.</v>
+      </c>
+      <c r="R18" t="str">
         <v>Baja</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R18"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A22"/>
   <cols>
     <col min="1" max="1" width="110.83203125" customWidth="1"/>
   </cols>
@@ -1072,82 +1464,97 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>3. Columnas &lt;gas&gt;_min y &lt;gas&gt;_max: rango del valor medido (inclusive). Puede llenar solo el mínimo, solo el máximo o ambos.</v>
+        <v xml:space="preserve">   Varias filas con el mismo diagnóstico funcionan como alternativas ("o"): si se cumple cualquiera, se muestra una vez.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>4. Columna "codigo": código que imprime el analizador (ej. E01). Varios códigos separados por coma.</v>
+        <v>3. Columnas &lt;gas&gt;_min y &lt;gas&gt;_max: rango del valor medido (inclusive). Puede llenar solo el mínimo, solo el máximo o ambos.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v xml:space="preserve">   Si una regla tiene código y rangos, deben cumplirse ambos.</v>
+        <v>4. Columna "codigo": código que imprime el analizador (ej. E01). Varios códigos separados por coma.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>5. "diagnostico" es obligatorio. "causas" y "recomendacion" son el detalle que verá el cliente.</v>
+        <v xml:space="preserve">   Si una regla tiene código y rangos, deben cumplirse ambos.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>6. "severidad": Alta, Media o Baja. Los resultados se ordenan de mayor a menor severidad.</v>
+        <v>5. "diagnostico" es obligatorio. "causas" y "recomendacion" son el detalle que verá el cliente.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>7. Use punto o coma como separador decimal.</v>
+        <v>6. "severidad": Alta, Media o Baja. Los resultados se ordenan de mayor a menor severidad.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>8. Guarde el archivo y cárguelo en la app con el botón "Cargar reglas (Excel)".</v>
+        <v>7. Use punto o coma como separador decimal.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>8. Guarde el archivo y cárguelo en la app con el botón "Cargar reglas (Excel)".</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Unidades</v>
+        <v>9. Las reglas base asumen gasolina, prueba en ralentí (máx. 1200 rpm) y motor a temperatura de operación.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CO: %</v>
+        <v xml:space="preserve">   Lambda (λ) se calcula automáticamente si el equipo no lo entrega.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>HC: ppm</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CO2: %</v>
+        <v>Unidades</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>O2: %</v>
+        <v>CO: %</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>NOx: ppm</v>
+        <v>HC: ppm</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>CO2: %</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>O2: %</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>NOx: ppm</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
         <v>Lambda: sin unidad</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adaptar al analizador del cliente (CO 0-10000 ppm, HC 0-1000 ppm)
- Avisos cuando CO o HC están en el máximo del equipo (R16, R17); con el CO
  saturado ya no se diagnostica catalizador en vez de mezcla rica
- Bordes de reglas exclusivos: sin huecos ni diagnósticos contradictorios con
  valores redondos (5000 ppm, 300 ppm, λ 0,970). Barrido: 0 contradicciones
- Lambda redondeado en el motor (lambdaForRules), igual en app y pruebas
- CO en ppm por defecto; el reporte muestra la lectura como se ingresó
- docs/REGLAS.md: sección del equipo del cliente

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantilla/reglas_ejemplo.xlsx
+++ b/plantilla/reglas_ejemplo.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:R21"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -540,10 +540,10 @@
         <v/>
       </c>
       <c r="C3">
-        <v>0.51</v>
+        <v>0.5001</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>0.9999</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -590,19 +590,19 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>R03</v>
+        <v>R02B</v>
       </c>
       <c r="B4" t="str">
         <v/>
       </c>
-      <c r="C4" t="str">
-        <v/>
+      <c r="C4">
+        <v>1.0001</v>
       </c>
       <c r="D4">
-        <v>0.5</v>
-      </c>
-      <c r="E4">
-        <v>101</v>
+        <v>3</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
       </c>
       <c r="F4">
         <v>400</v>
@@ -646,25 +646,25 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>R04</v>
+        <v>R03</v>
       </c>
       <c r="B5" t="str">
         <v/>
       </c>
-      <c r="C5">
-        <v>1</v>
+      <c r="C5" t="str">
+        <v/>
       </c>
       <c r="D5">
-        <v>2.99</v>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v/>
+        <v>0.5</v>
+      </c>
+      <c r="E5">
+        <v>100.0001</v>
+      </c>
+      <c r="F5">
+        <v>400</v>
+      </c>
+      <c r="G5">
+        <v>12</v>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -681,20 +681,20 @@
       <c r="L5" t="str">
         <v/>
       </c>
-      <c r="M5" t="str">
-        <v/>
+      <c r="M5">
+        <v>0.97</v>
       </c>
       <c r="N5">
-        <v>0.97</v>
+        <v>1.03</v>
       </c>
       <c r="O5" t="str">
-        <v>Mezcla rica</v>
+        <v>Catalizador con baja eficiencia</v>
       </c>
       <c r="P5" t="str">
-        <v>Exceso de combustible: CO alto con O₂ bajo. Posibles causas: sensor de oxígeno sesgado o lento, sensor de temperatura del refrigerante indicando motor frío, presión de combustible alta (regulador), inyectores goteando, canister EVAP saturado, válvula PCV obstruida, filtro de aire sucio (motores con sensor MAP).</v>
+        <v>La mezcla es correcta (λ ≈ 1) y la combustión eficiente (CO₂ normal), pero salen CO o HC por encima de lo esperado: el catalizador no está convirtiendo los gases (desgastado, contaminado por aceite o anticongelante, o no alcanza su temperatura). En vehículos sin catalizador estos valores pueden ser normales.</v>
       </c>
       <c r="Q5" t="str">
-        <v>Revisar con escáner los ajustes de combustible (fuel trims) y los sensores de O₂, ECT y MAP/MAF. Medir la presión de combustible y probar el regulador e inyectores. Revisar PCV, canister y filtro de aire.</v>
+        <v>Verificar que el vehículo tenga catalizador y que el motor esté caliente. Medir la temperatura a la entrada y salida del catalizador (la salida debe estar más caliente). Si no convierte, reemplazarlo y corregir la causa (consumo de aceite, fallas de encendido).</v>
       </c>
       <c r="R5" t="str">
         <v>Media</v>
@@ -702,16 +702,16 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>R05</v>
+        <v>R04</v>
       </c>
       <c r="B6" t="str">
         <v/>
       </c>
       <c r="C6">
-        <v>3</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>2.9999</v>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -741,39 +741,39 @@
         <v/>
       </c>
       <c r="N6">
-        <v>0.97</v>
+        <v>0.9699</v>
       </c>
       <c r="O6" t="str">
-        <v>Mezcla muy rica</v>
+        <v>Mezcla rica</v>
       </c>
       <c r="P6" t="str">
-        <v>Gran exceso de combustible (CO muy alto con O₂ bajo): inyector goteando o pegado abierto, regulador de presión dañado, sensor ECT o de O₂ defectuoso, combustible en el aceite del cárter. En carburados: flotador hundido o chiclé desgastado.</v>
+        <v>Exceso de combustible: CO alto con O₂ bajo. Posibles causas: sensor de oxígeno sesgado o lento, sensor de temperatura del refrigerante indicando motor frío, presión de combustible alta (regulador), inyectores goteando, canister EVAP saturado, válvula PCV obstruida, filtro de aire sucio (motores con sensor MAP).</v>
       </c>
       <c r="Q6" t="str">
-        <v>Corregir de inmediato: consume combustible en exceso y daña el catalizador. Medir presión de combustible, probar estanqueidad de inyectores, revisar sensores con escáner y oler el aceite por dilución con gasolina (cambiarlo si está contaminado).</v>
+        <v>Revisar con escáner los ajustes de combustible (fuel trims) y los sensores de O₂, ECT y MAP/MAF. Medir la presión de combustible y probar el regulador e inyectores. Revisar PCV, canister y filtro de aire.</v>
       </c>
       <c r="R6" t="str">
-        <v>Alta</v>
+        <v>Media</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>R06</v>
+        <v>R05</v>
       </c>
       <c r="B7" t="str">
         <v/>
       </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7">
-        <v>0.99</v>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
       </c>
       <c r="E7" t="str">
         <v/>
       </c>
-      <c r="F7">
-        <v>299</v>
+      <c r="F7" t="str">
+        <v/>
       </c>
       <c r="G7" t="str">
         <v/>
@@ -781,8 +781,8 @@
       <c r="H7" t="str">
         <v/>
       </c>
-      <c r="I7">
-        <v>2</v>
+      <c r="I7" t="str">
+        <v/>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -796,25 +796,25 @@
       <c r="M7" t="str">
         <v/>
       </c>
-      <c r="N7" t="str">
-        <v/>
+      <c r="N7">
+        <v>0.9699</v>
       </c>
       <c r="O7" t="str">
-        <v>Mezcla pobre</v>
+        <v>Mezcla muy rica</v>
       </c>
       <c r="P7" t="str">
-        <v>Falta de combustible o exceso de aire: O₂ alto con CO bajo. Posibles causas: entrada de aire falso (fuga de vacío, mangueras, empaque del múltiple de admisión), inyectores obstruidos, presión o caudal de combustible bajos, sensor MAF sucio.</v>
+        <v>Gran exceso de combustible (CO muy alto con O₂ bajo): inyector goteando o pegado abierto, regulador de presión dañado, sensor ECT o de O₂ defectuoso, combustible en el aceite del cárter. En carburados: flotador hundido o chiclé desgastado.</v>
       </c>
       <c r="Q7" t="str">
-        <v>Buscar fugas de vacío (prueba de humo o con limpiador de carburador y RPM), limpiar inyectores y sensor MAF, medir presión y caudal de la bomba de combustible y revisar el filtro de combustible.</v>
+        <v>Corregir de inmediato: consume combustible en exceso y daña el catalizador. Medir presión de combustible, probar estanqueidad de inyectores, revisar sensores con escáner y oler el aceite por dilución con gasolina (cambiarlo si está contaminado).</v>
       </c>
       <c r="R7" t="str">
-        <v>Media</v>
+        <v>Alta</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>R06B</v>
+        <v>R06</v>
       </c>
       <c r="B8" t="str">
         <v/>
@@ -823,13 +823,13 @@
         <v/>
       </c>
       <c r="D8">
-        <v>0.99</v>
+        <v>0.9999</v>
       </c>
       <c r="E8" t="str">
         <v/>
       </c>
       <c r="F8">
-        <v>299</v>
+        <v>299.9999</v>
       </c>
       <c r="G8" t="str">
         <v/>
@@ -837,8 +837,8 @@
       <c r="H8" t="str">
         <v/>
       </c>
-      <c r="I8" t="str">
-        <v/>
+      <c r="I8">
+        <v>2</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -849,8 +849,8 @@
       <c r="L8" t="str">
         <v/>
       </c>
-      <c r="M8">
-        <v>1.05</v>
+      <c r="M8" t="str">
+        <v/>
       </c>
       <c r="N8" t="str">
         <v/>
@@ -870,22 +870,22 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>R07</v>
+        <v>R06B</v>
       </c>
       <c r="B9" t="str">
         <v/>
       </c>
-      <c r="C9">
-        <v>0.5</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9">
-        <v>300</v>
-      </c>
-      <c r="F9" t="str">
-        <v/>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9">
+        <v>0.9999</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9">
+        <v>299.9999</v>
       </c>
       <c r="G9" t="str">
         <v/>
@@ -893,8 +893,8 @@
       <c r="H9" t="str">
         <v/>
       </c>
-      <c r="I9">
-        <v>2</v>
+      <c r="I9" t="str">
+        <v/>
       </c>
       <c r="J9" t="str">
         <v/>
@@ -905,34 +905,34 @@
       <c r="L9" t="str">
         <v/>
       </c>
-      <c r="M9" t="str">
-        <v/>
+      <c r="M9">
+        <v>1.05</v>
       </c>
       <c r="N9" t="str">
         <v/>
       </c>
       <c r="O9" t="str">
-        <v>Falla de encendido (cilindro que no quema)</v>
+        <v>Mezcla pobre</v>
       </c>
       <c r="P9" t="str">
-        <v>HC muy alto junto con O₂ y CO altos: un cilindro no quema la mezcla y sale combustible crudo; la computadora interpreta el oxígeno sobrante como mezcla pobre y enriquece. Posibles causas: bujías gastadas o sucias, cables o bobinas defectuosos, inyector de ese cilindro sin pulverizar.</v>
+        <v>Falta de combustible o exceso de aire: O₂ alto con CO bajo. Posibles causas: entrada de aire falso (fuga de vacío, mangueras, empaque del múltiple de admisión), inyectores obstruidos, presión o caudal de combustible bajos, sensor MAF sucio.</v>
       </c>
       <c r="Q9" t="str">
-        <v>Revisar con escáner los contadores de fallas por cilindro (misfire). Inspeccionar bujías, cables y bobinas; intercambiar bobinas entre cilindros para ubicar la falla. Si persiste, prueba de compresión.</v>
+        <v>Buscar fugas de vacío (prueba de humo o con limpiador de carburador y RPM), limpiar inyectores y sensor MAF, medir presión y caudal de la bomba de combustible y revisar el filtro de combustible.</v>
       </c>
       <c r="R9" t="str">
-        <v>Alta</v>
+        <v>Media</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>R07B</v>
+        <v>R07</v>
       </c>
       <c r="B10" t="str">
         <v/>
       </c>
       <c r="C10">
-        <v>1.51</v>
+        <v>0.5001</v>
       </c>
       <c r="D10" t="str">
         <v/>
@@ -950,7 +950,7 @@
         <v/>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -982,16 +982,16 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>R08</v>
+        <v>R07B</v>
       </c>
       <c r="B11" t="str">
         <v/>
       </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11">
-        <v>0.49</v>
+      <c r="C11">
+        <v>1.5001</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
       </c>
       <c r="E11">
         <v>300</v>
@@ -1006,7 +1006,7 @@
         <v/>
       </c>
       <c r="I11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -1024,13 +1024,13 @@
         <v/>
       </c>
       <c r="O11" t="str">
-        <v>Falla por mezcla muy pobre</v>
+        <v>Falla de encendido (cilindro que no quema)</v>
       </c>
       <c r="P11" t="str">
-        <v>HC alto con O₂ muy alto y CO muy bajo: la mezcla es tan pobre que la llama no la quema por completo (falla por mezcla pobre). Posibles causas: fuga de vacío grande, inyectores obstruidos, presión de combustible muy baja, sensor MAF defectuoso.</v>
+        <v>HC muy alto junto con O₂ y CO altos: un cilindro no quema la mezcla y sale combustible crudo; la computadora interpreta el oxígeno sobrante como mezcla pobre y enriquece. Posibles causas: bujías gastadas o sucias, cables o bobinas defectuosos, inyector de ese cilindro sin pulverizar.</v>
       </c>
       <c r="Q11" t="str">
-        <v>Buscar fugas de vacío grandes, medir presión y caudal de combustible, limpiar o probar inyectores y el sensor MAF. Verificar también que la sonda del analizador no tome aire (ver muestra diluida).</v>
+        <v>Revisar con escáner los contadores de fallas por cilindro (misfire). Inspeccionar bujías, cables y bobinas; intercambiar bobinas entre cilindros para ubicar la falla. Si persiste, prueba de compresión.</v>
       </c>
       <c r="R11" t="str">
         <v>Alta</v>
@@ -1038,7 +1038,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>R09</v>
+        <v>R08</v>
       </c>
       <c r="B12" t="str">
         <v/>
@@ -1047,7 +1047,7 @@
         <v/>
       </c>
       <c r="D12">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="E12">
         <v>300</v>
@@ -1061,11 +1061,11 @@
       <c r="H12" t="str">
         <v/>
       </c>
-      <c r="I12" t="str">
-        <v/>
-      </c>
-      <c r="J12">
-        <v>1.99</v>
+      <c r="I12">
+        <v>2</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -1080,36 +1080,36 @@
         <v/>
       </c>
       <c r="O12" t="str">
-        <v>HC alto sin problema de mezcla: compresión, aceite o puesta a punto</v>
+        <v>Falla por mezcla muy pobre</v>
       </c>
       <c r="P12" t="str">
-        <v>Mezcla normal (ni CO ni O₂ altos) pero HC alto: el combustible no termina de quemarse por baja compresión (anillos, válvulas quemadas o mal asentadas), paso de aceite a la cámara (guías o sellos de válvula, anillos), válvula EGR abierta en ralentí o avance de encendido excesivo.</v>
+        <v>HC alto con O₂ muy alto y CO muy bajo: la mezcla es tan pobre que la llama no la quema por completo (falla por mezcla pobre). Posibles causas: fuga de vacío grande, inyectores obstruidos, presión de combustible muy baja, sensor MAF defectuoso.</v>
       </c>
       <c r="Q12" t="str">
-        <v>Hacer prueba de compresión seca y húmeda o de fugas de cilindro, revisar humo azul y consumo de aceite, verificar que la EGR cierre en ralentí y comprobar el avance de encendido.</v>
+        <v>Buscar fugas de vacío grandes, medir presión y caudal de combustible, limpiar o probar inyectores y el sensor MAF. Verificar también que la sonda del analizador no tome aire (ver muestra diluida).</v>
       </c>
       <c r="R12" t="str">
-        <v>Media</v>
+        <v>Alta</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>R10</v>
+        <v>R09</v>
       </c>
       <c r="B13" t="str">
         <v/>
       </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
-      <c r="E13" t="str">
-        <v/>
-      </c>
-      <c r="F13">
-        <v>299</v>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13">
+        <v>1.5</v>
+      </c>
+      <c r="E13">
+        <v>300</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
       </c>
       <c r="G13" t="str">
         <v/>
@@ -1117,11 +1117,11 @@
       <c r="H13" t="str">
         <v/>
       </c>
-      <c r="I13">
-        <v>2</v>
-      </c>
-      <c r="J13" t="str">
-        <v/>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13">
+        <v>1.9999</v>
       </c>
       <c r="K13" t="str">
         <v/>
@@ -1136,13 +1136,13 @@
         <v/>
       </c>
       <c r="O13" t="str">
-        <v>CO y O₂ altos a la vez</v>
+        <v>HC alto sin problema de mezcla: compresión, aceite o puesta a punto</v>
       </c>
       <c r="P13" t="str">
-        <v>En una combustión normal no pueden estar ambos altos. Indica aire que entra al escape antes de la sonda de oxígeno (fuga en múltiple o tubo de escape), sistema de inyección de aire secundario activo, o mezcla desigual entre cilindros (un inyector goteando y otro obstruido).</v>
+        <v>Mezcla normal (ni CO ni O₂ altos) pero HC alto: el combustible no termina de quemarse por baja compresión (anillos, válvulas quemadas o mal asentadas), paso de aceite a la cámara (guías o sellos de válvula, anillos), válvula EGR abierta en ralentí o avance de encendido excesivo.</v>
       </c>
       <c r="Q13" t="str">
-        <v>Revisar fugas en el múltiple y el tubo de escape antes de la sonda de O₂, verificar el sistema de aire secundario si lo tiene, y hacer prueba de balance de inyectores.</v>
+        <v>Hacer prueba de compresión seca y húmeda o de fugas de cilindro, revisar humo azul y consumo de aceite, verificar que la EGR cierre en ralentí y comprobar el avance de encendido.</v>
       </c>
       <c r="R13" t="str">
         <v>Media</v>
@@ -1150,13 +1150,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>R11</v>
+        <v>R10</v>
       </c>
       <c r="B14" t="str">
         <v/>
       </c>
-      <c r="C14" t="str">
-        <v/>
+      <c r="C14">
+        <v>1</v>
       </c>
       <c r="D14" t="str">
         <v/>
@@ -1165,16 +1165,16 @@
         <v/>
       </c>
       <c r="F14">
-        <v>300</v>
+        <v>299.9999</v>
       </c>
       <c r="G14" t="str">
         <v/>
       </c>
-      <c r="H14">
-        <v>10</v>
+      <c r="H14" t="str">
+        <v/>
       </c>
       <c r="I14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J14" t="str">
         <v/>
@@ -1192,21 +1192,21 @@
         <v/>
       </c>
       <c r="O14" t="str">
-        <v>Muestra diluida: prueba no válida</v>
+        <v>CO y O₂ altos a la vez</v>
       </c>
       <c r="P14" t="str">
-        <v>CO₂ muy bajo con O₂ alto y HC normal: el analizador está midiendo aire mezclado con los gases. Sonda insertada poco profundo, fuga en el sistema de escape, o manguera o filtro del analizador con fugas.</v>
+        <v>En una combustión normal no pueden estar ambos altos. Indica aire que entra al escape antes de la sonda de oxígeno (fuga en múltiple o tubo de escape), sistema de inyección de aire secundario activo, o mezcla desigual entre cilindros (un inyector goteando y otro obstruido).</v>
       </c>
       <c r="Q14" t="str">
-        <v>Insertar la sonda al menos 30 cm dentro del tubo de escape, revisar fugas del escape y de la manguera del analizador, y repetir la medición antes de interpretar los demás resultados.</v>
+        <v>Revisar fugas en el múltiple y el tubo de escape antes de la sonda de O₂, verificar el sistema de aire secundario si lo tiene, y hacer prueba de balance de inyectores.</v>
       </c>
       <c r="R14" t="str">
-        <v>Alta</v>
+        <v>Media</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>R12</v>
+        <v>R11</v>
       </c>
       <c r="B15" t="str">
         <v/>
@@ -1220,17 +1220,17 @@
       <c r="E15" t="str">
         <v/>
       </c>
-      <c r="F15" t="str">
-        <v/>
+      <c r="F15">
+        <v>300</v>
       </c>
       <c r="G15" t="str">
         <v/>
       </c>
       <c r="H15">
-        <v>12.49</v>
-      </c>
-      <c r="I15" t="str">
-        <v/>
+        <v>10</v>
+      </c>
+      <c r="I15">
+        <v>4</v>
       </c>
       <c r="J15" t="str">
         <v/>
@@ -1241,28 +1241,28 @@
       <c r="L15" t="str">
         <v/>
       </c>
-      <c r="M15">
-        <v>0.97</v>
-      </c>
-      <c r="N15">
-        <v>1.03</v>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
       </c>
       <c r="O15" t="str">
-        <v>Combustión ineficiente (CO₂ bajo)</v>
+        <v>Muestra diluida: prueba no válida</v>
       </c>
       <c r="P15" t="str">
-        <v>Mezcla correcta pero CO₂ bajo: la combustión no es completa. Posibles causas: puesta a punto incorrecta (avance), válvula EGR abierta en ralentí, baja compresión, o analizador descalibrado o con fugas en la sonda.</v>
+        <v>CO₂ muy bajo con O₂ alto y HC normal: el analizador está midiendo aire mezclado con los gases. Sonda insertada poco profundo, fuga en el sistema de escape, o manguera o filtro del analizador con fugas.</v>
       </c>
       <c r="Q15" t="str">
-        <v>Verificar el avance de encendido y la EGR, hacer prueba de compresión y comprobar la calibración del analizador.</v>
+        <v>Insertar la sonda al menos 30 cm dentro del tubo de escape, revisar fugas del escape y de la manguera del analizador, y repetir la medición antes de interpretar los demás resultados.</v>
       </c>
       <c r="R15" t="str">
-        <v>Media</v>
+        <v>Alta</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>R13</v>
+        <v>R12</v>
       </c>
       <c r="B16" t="str">
         <v/>
@@ -1282,8 +1282,8 @@
       <c r="G16" t="str">
         <v/>
       </c>
-      <c r="H16" t="str">
-        <v/>
+      <c r="H16">
+        <v>12.4999</v>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -1291,26 +1291,26 @@
       <c r="J16" t="str">
         <v/>
       </c>
-      <c r="K16">
-        <v>1000</v>
+      <c r="K16" t="str">
+        <v/>
       </c>
       <c r="L16" t="str">
         <v/>
       </c>
-      <c r="M16" t="str">
-        <v/>
-      </c>
-      <c r="N16" t="str">
-        <v/>
+      <c r="M16">
+        <v>0.97</v>
+      </c>
+      <c r="N16">
+        <v>1.03</v>
       </c>
       <c r="O16" t="str">
-        <v>NOx elevado (temperatura de combustión alta)</v>
+        <v>Combustión ineficiente (CO₂ bajo)</v>
       </c>
       <c r="P16" t="str">
-        <v>Temperatura o presión de combustión excesivas: válvula EGR obstruida o inoperante, mezcla pobre, avance de encendido excesivo, carbonilla en pistones o válvulas, sistema de enfriamiento deficiente, combustible de bajo octanaje o sensor de detonación inoperante.</v>
+        <v>Mezcla correcta pero CO₂ bajo: la combustión no es completa. Posibles causas: puesta a punto incorrecta (avance), válvula EGR abierta en ralentí, baja compresión, o analizador descalibrado o con fugas en la sonda.</v>
       </c>
       <c r="Q16" t="str">
-        <v>Revisar y limpiar la válvula EGR y sus conductos, verificar el avance de encendido y el sensor de detonación, descarbonizar el motor y revisar el sistema de enfriamiento.</v>
+        <v>Verificar el avance de encendido y la EGR, hacer prueba de compresión y comprobar la calibración del analizador.</v>
       </c>
       <c r="R16" t="str">
         <v>Media</v>
@@ -1318,7 +1318,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>R14</v>
+        <v>R13</v>
       </c>
       <c r="B17" t="str">
         <v/>
@@ -1326,14 +1326,14 @@
       <c r="C17" t="str">
         <v/>
       </c>
-      <c r="D17">
-        <v>1</v>
+      <c r="D17" t="str">
+        <v/>
       </c>
       <c r="E17" t="str">
         <v/>
       </c>
-      <c r="F17">
-        <v>300</v>
+      <c r="F17" t="str">
+        <v/>
       </c>
       <c r="G17" t="str">
         <v/>
@@ -1347,34 +1347,34 @@
       <c r="J17" t="str">
         <v/>
       </c>
-      <c r="K17" t="str">
-        <v/>
+      <c r="K17">
+        <v>1000</v>
       </c>
       <c r="L17" t="str">
         <v/>
       </c>
-      <c r="M17">
-        <v>1.031</v>
-      </c>
-      <c r="N17">
-        <v>1.049</v>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
       </c>
       <c r="O17" t="str">
-        <v>Mezcla ligeramente pobre</v>
+        <v>NOx elevado (temperatura de combustión alta)</v>
       </c>
       <c r="P17" t="str">
-        <v>Lambda algo por encima de 1. Puede ser la oscilación normal del control de mezcla en el momento de la medición, o una pequeña entrada de aire falso, inyectores algo sucios o un sensor de oxígeno lento.</v>
+        <v>Temperatura o presión de combustión excesivas: válvula EGR obstruida o inoperante, mezcla pobre, avance de encendido excesivo, carbonilla en pistones o válvulas, sistema de enfriamiento deficiente, combustible de bajo octanaje o sensor de detonación inoperante.</v>
       </c>
       <c r="Q17" t="str">
-        <v>Repetir la medición con el motor estabilizado. Si se mantiene, revisar con escáner los ajustes de combustible (fuel trims) y buscar pequeñas fugas de vacío.</v>
+        <v>Revisar y limpiar la válvula EGR y sus conductos, verificar el avance de encendido y el sensor de detonación, descarbonizar el motor y revisar el sistema de enfriamiento.</v>
       </c>
       <c r="R17" t="str">
-        <v>Baja</v>
+        <v>Media</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>R15</v>
+        <v>R14</v>
       </c>
       <c r="B18" t="str">
         <v/>
@@ -1383,13 +1383,13 @@
         <v/>
       </c>
       <c r="D18">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="E18" t="str">
         <v/>
       </c>
-      <c r="F18" t="str">
-        <v/>
+      <c r="F18">
+        <v>300</v>
       </c>
       <c r="G18" t="str">
         <v/>
@@ -1400,8 +1400,8 @@
       <c r="I18" t="str">
         <v/>
       </c>
-      <c r="J18">
-        <v>1.5</v>
+      <c r="J18" t="str">
+        <v/>
       </c>
       <c r="K18" t="str">
         <v/>
@@ -1410,27 +1410,195 @@
         <v/>
       </c>
       <c r="M18">
-        <v>0.95</v>
+        <v>1.0301</v>
       </c>
       <c r="N18">
-        <v>0.969</v>
+        <v>1.0499</v>
       </c>
       <c r="O18" t="str">
-        <v>Mezcla ligeramente rica</v>
+        <v>Mezcla ligeramente pobre</v>
       </c>
       <c r="P18" t="str">
-        <v>Lambda algo por debajo de 1. Puede ser la oscilación normal del control de mezcla, o un leve exceso de combustible: sensor de oxígeno lento, filtro de aire sucio o canister EVAP purgando.</v>
+        <v>Lambda algo por encima de 1. Puede ser la oscilación normal del control de mezcla en el momento de la medición, o una pequeña entrada de aire falso, inyectores algo sucios o un sensor de oxígeno lento.</v>
       </c>
       <c r="Q18" t="str">
-        <v>Repetir la medición con el motor estabilizado. Si se mantiene, revisar con escáner los ajustes de combustible, el sensor de oxígeno y el filtro de aire.</v>
+        <v>Repetir la medición con el motor estabilizado. Si se mantiene, revisar con escáner los ajustes de combustible (fuel trims) y buscar pequeñas fugas de vacío.</v>
       </c>
       <c r="R18" t="str">
         <v>Baja</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>R15</v>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19">
+        <v>0.9999</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19">
+        <v>1.5</v>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19">
+        <v>0.95</v>
+      </c>
+      <c r="N19">
+        <v>0.9699</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Mezcla ligeramente rica</v>
+      </c>
+      <c r="P19" t="str">
+        <v>Lambda algo por debajo de 1. Puede ser la oscilación normal del control de mezcla, o un leve exceso de combustible: sensor de oxígeno lento, filtro de aire sucio o canister EVAP purgando.</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>Repetir la medición con el motor estabilizado. Si se mantiene, revisar con escáner los ajustes de combustible, el sensor de oxígeno y el filtro de aire.</v>
+      </c>
+      <c r="R19" t="str">
+        <v>Baja</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>R16</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v>CO en el máximo del equipo (10 000 ppm)</v>
+      </c>
+      <c r="P20" t="str">
+        <v>El analizador mide CO hasta 10 000 ppm (1 %). Con la lectura en el tope, el CO real puede ser mayor: la mezcla probablemente es rica y el lambda calculado sale más alto (más cercano a 1) de lo real.</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>Tratar como mezcla rica: revisar presión de combustible, inyectores y sensores (O₂, temperatura, MAP/MAF). Para cuantificar el CO real se necesita un analizador con rango de al menos 10 %.</v>
+      </c>
+      <c r="R20" t="str">
+        <v>Alta</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>R17</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21">
+        <v>1000</v>
+      </c>
+      <c r="F21">
+        <v>1000</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v>HC en el máximo del equipo (1000 ppm)</v>
+      </c>
+      <c r="P21" t="str">
+        <v>El analizador mide HC hasta 1000 ppm. Con la lectura en el tope, el HC real puede ser bastante mayor, lo que es típico de una falla de encendido o de un cilindro que no quema.</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>Revisar bujías, cables, bobinas y contadores de fallas por cilindro con escáner. Para cuantificar el HC real se necesita un analizador de mayor rango.</v>
+      </c>
+      <c r="R21" t="str">
+        <v>Alta</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>